<commit_message>
fix: update student spreadsheet template
</commit_message>
<xml_diff>
--- a/public/student_template.xlsx
+++ b/public/student_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dan/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shaynesidman/projects/mhd/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5745453-EE54-8440-9E82-6E8066158FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548742BD-1EB4-C048-85AC-EC669B0F819E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Student" sheetId="1" r:id="rId1"/>
@@ -45,9 +45,6 @@
     <t>teacherEmail</t>
   </si>
   <si>
-    <t>projectId</t>
-  </si>
-  <si>
     <t>teamProject</t>
   </si>
   <si>
@@ -58,6 +55,9 @@
   </si>
   <si>
     <t>title</t>
+  </si>
+  <si>
+    <t>projectIntId</t>
   </si>
 </sst>
 </file>
@@ -80,11 +80,13 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -391,19 +393,19 @@
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1">

</xml_diff>